<commit_message>
Add the architecture diagram, the UC-02 activity diagram and PDF copies of the requirements table and UC-02 spec, and update the WBS and README to match.
</commit_message>
<xml_diff>
--- a/4-SRS-and-WBS/WBS.xlsx
+++ b/4-SRS-and-WBS/WBS.xlsx
@@ -1048,9 +1048,9 @@
       <c r="F20" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>